<commit_message>
Reduce memory by encoding equivalence classes using cycles.
</commit_message>
<xml_diff>
--- a/Prefixes.xlsx
+++ b/Prefixes.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3869509-3D65-4367-B5C0-31E769FF9C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AD8596-6F59-4F20-9B67-EC9A75E21022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Symmetric" sheetId="1" r:id="rId1"/>
-    <sheet name="All" sheetId="3" r:id="rId2"/>
+    <sheet name="2unsym" sheetId="3" r:id="rId1"/>
+    <sheet name="2sym" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -443,130 +443,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFA2CA3B-EC37-4E3A-9860-8E9F3C166319}">
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.33203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="2">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2">
-        <v>6</v>
-      </c>
-      <c r="E1" s="2">
-        <v>8</v>
-      </c>
-      <c r="F1" s="2">
-        <v>10</v>
-      </c>
-      <c r="G1" s="2">
-        <v>12</v>
-      </c>
-      <c r="H1" s="2">
-        <v>14</v>
-      </c>
-      <c r="I1" s="2">
-        <v>16</v>
-      </c>
-      <c r="J1" s="2">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1">
-        <v>4</v>
-      </c>
-      <c r="E3" s="1">
-        <v>5</v>
-      </c>
-      <c r="F3" s="1">
-        <v>13</v>
-      </c>
-      <c r="G3" s="1">
-        <v>15</v>
-      </c>
-      <c r="H3" s="1">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1">
-        <v>2</v>
-      </c>
-      <c r="D4" s="1">
-        <v>4</v>
-      </c>
-      <c r="E4" s="1">
-        <v>5</v>
-      </c>
-      <c r="F4" s="1">
-        <v>13</v>
-      </c>
-      <c r="G4" s="1">
-        <v>15</v>
-      </c>
-      <c r="H4" s="1">
-        <v>41</v>
-      </c>
-      <c r="I4" s="1">
-        <v>36</v>
-      </c>
-      <c r="J4" s="1">
-        <v>118</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4722944D-AFB6-47E1-8B0E-05331FFCD6B7}">
   <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -729,6 +605,145 @@
       <c r="L4" s="1">
         <v>70</v>
       </c>
+      <c r="M4" s="1">
+        <v>212</v>
+      </c>
+      <c r="N4" s="1">
+        <v>136</v>
+      </c>
+      <c r="O4" s="1">
+        <v>494</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFA2CA3B-EC37-4E3A-9860-8E9F3C166319}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.33203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2">
+        <v>14</v>
+      </c>
+      <c r="I1" s="2">
+        <v>16</v>
+      </c>
+      <c r="J1" s="2">
+        <v>18</v>
+      </c>
+      <c r="K1" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1">
+        <v>4</v>
+      </c>
+      <c r="E2" s="1">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4</v>
+      </c>
+      <c r="E3" s="1">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1">
+        <v>13</v>
+      </c>
+      <c r="G3" s="1">
+        <v>15</v>
+      </c>
+      <c r="H3" s="1">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>4</v>
+      </c>
+      <c r="E4" s="1">
+        <v>5</v>
+      </c>
+      <c r="F4" s="1">
+        <v>13</v>
+      </c>
+      <c r="G4" s="1">
+        <v>15</v>
+      </c>
+      <c r="H4" s="1">
+        <v>41</v>
+      </c>
+      <c r="I4" s="1">
+        <v>36</v>
+      </c>
+      <c r="J4" s="1">
+        <v>118</v>
+      </c>
+      <c r="K4" s="1">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Support generating 3-layer prefixes using the prefix graph.
</commit_message>
<xml_diff>
--- a/Prefixes.xlsx
+++ b/Prefixes.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AD8596-6F59-4F20-9B67-EC9A75E21022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D732EF2F-4AE0-49B4-8B45-B89FB3F9698C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="2unsym" sheetId="3" r:id="rId1"/>
     <sheet name="2sym" sheetId="1" r:id="rId2"/>
+    <sheet name="3sym" sheetId="5" r:id="rId3"/>
+    <sheet name="3unsym" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="4">
   <si>
     <t>Subsumption</t>
   </si>
@@ -664,6 +666,136 @@
         <v>20</v>
       </c>
     </row>
+    <row r="2" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1">
+        <v>4</v>
+      </c>
+      <c r="E2" s="1">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4</v>
+      </c>
+      <c r="E3" s="1">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1">
+        <v>13</v>
+      </c>
+      <c r="G3" s="1">
+        <v>15</v>
+      </c>
+      <c r="H3" s="1">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>4</v>
+      </c>
+      <c r="E4" s="1">
+        <v>5</v>
+      </c>
+      <c r="F4" s="1">
+        <v>13</v>
+      </c>
+      <c r="G4" s="1">
+        <v>15</v>
+      </c>
+      <c r="H4" s="1">
+        <v>41</v>
+      </c>
+      <c r="I4" s="1">
+        <v>36</v>
+      </c>
+      <c r="J4" s="1">
+        <v>118</v>
+      </c>
+      <c r="K4" s="1">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FDE5C09-6236-4F3A-B612-F2350551A5C2}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.33203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2">
+        <v>14</v>
+      </c>
+      <c r="I1" s="2">
+        <v>16</v>
+      </c>
+      <c r="J1" s="2">
+        <v>18</v>
+      </c>
+      <c r="K1" s="2">
+        <v>20</v>
+      </c>
+    </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
@@ -672,16 +804,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" s="1">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -695,19 +824,10 @@
         <v>2</v>
       </c>
       <c r="D3" s="1">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E3" s="1">
-        <v>5</v>
-      </c>
-      <c r="F3" s="1">
-        <v>13</v>
-      </c>
-      <c r="G3" s="1">
-        <v>15</v>
-      </c>
-      <c r="H3" s="1">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -721,28 +841,164 @@
         <v>2</v>
       </c>
       <c r="D4" s="1">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1">
+        <v>47</v>
+      </c>
+      <c r="F4" s="1">
+        <v>504</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1632</v>
+      </c>
+      <c r="H4" s="1">
+        <v>24117</v>
+      </c>
+      <c r="I4" s="1">
+        <v>56884</v>
+      </c>
+      <c r="J4" s="1">
+        <v>1004741</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD7D369D-3D6A-4BDB-B488-E0821FACF492}">
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.33203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2">
         <v>4</v>
       </c>
+      <c r="E1" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1" s="2">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2">
+        <v>7</v>
+      </c>
+      <c r="H1" s="2">
+        <v>8</v>
+      </c>
+      <c r="I1" s="2">
+        <v>9</v>
+      </c>
+      <c r="J1" s="2">
+        <v>10</v>
+      </c>
+      <c r="K1" s="2">
+        <v>11</v>
+      </c>
+      <c r="L1" s="2">
+        <v>12</v>
+      </c>
+      <c r="M1" s="2">
+        <v>13</v>
+      </c>
+      <c r="N1" s="2">
+        <v>14</v>
+      </c>
+      <c r="O1" s="2">
+        <v>15</v>
+      </c>
+      <c r="P1" s="2">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="2">
+        <v>17</v>
+      </c>
+      <c r="R1" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1">
+        <v>29</v>
+      </c>
+      <c r="F3" s="1">
+        <v>55</v>
+      </c>
+      <c r="G3" s="1">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2</v>
+      </c>
       <c r="E4" s="1">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="F4" s="1">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="G4" s="1">
-        <v>15</v>
-      </c>
-      <c r="H4" s="1">
-        <v>41</v>
-      </c>
-      <c r="I4" s="1">
-        <v>36</v>
-      </c>
-      <c r="J4" s="1">
-        <v>118</v>
-      </c>
-      <c r="K4" s="1">
-        <v>89</v>
+        <v>489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add edges using output isomorphism.
</commit_message>
<xml_diff>
--- a/Prefixes.xlsx
+++ b/Prefixes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D732EF2F-4AE0-49B4-8B45-B89FB3F9698C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDB9E51-34BD-46F3-85C3-CA386E0C5129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="6">
   <si>
     <t>Subsumption</t>
   </si>
@@ -54,6 +54,12 @@
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>PG (IsoOutputs)</t>
+  </si>
+  <si>
+    <t>PG (IsoOutputs + OutputSubsets)</t>
   </si>
 </sst>
 </file>
@@ -754,10 +760,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FDE5C09-6236-4F3A-B612-F2350551A5C2}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="29.5" style="1" customWidth="1"/>
     <col min="2" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
@@ -860,6 +866,89 @@
       </c>
       <c r="J4" s="1">
         <v>1004741</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>8</v>
+      </c>
+      <c r="E5" s="1">
+        <v>27</v>
+      </c>
+      <c r="F5" s="1">
+        <v>316</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1101</v>
+      </c>
+      <c r="H5" s="1">
+        <v>15713</v>
+      </c>
+      <c r="I5" s="1">
+        <v>39757</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1">
+        <v>4</v>
+      </c>
+      <c r="E6" s="1">
+        <v>15</v>
+      </c>
+      <c r="F6" s="1">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B8" s="1">
+        <f>B4/B5</f>
+        <v>1</v>
+      </c>
+      <c r="C8" s="1">
+        <f t="shared" ref="C8:I8" si="0">C4/C5</f>
+        <v>2</v>
+      </c>
+      <c r="D8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.875</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.7407407407407407</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.5949367088607596</v>
+      </c>
+      <c r="G8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.4822888283378746</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.5348437599439955</v>
+      </c>
+      <c r="I8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.430792061775285</v>
       </c>
     </row>
   </sheetData>
@@ -869,7 +958,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD7D369D-3D6A-4BDB-B488-E0821FACF492}">
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
@@ -954,6 +1043,9 @@
       <c r="G2" s="1">
         <v>99</v>
       </c>
+      <c r="H2" s="1">
+        <v>68</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -999,6 +1091,38 @@
       </c>
       <c r="G4" s="1">
         <v>489</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1">
+        <v>14</v>
+      </c>
+      <c r="F5" s="1">
+        <v>31</v>
+      </c>
+      <c r="G5" s="1">
+        <v>290</v>
+      </c>
+      <c r="H5" s="1">
+        <v>760</v>
+      </c>
+      <c r="I5" s="1">
+        <v>7400</v>
+      </c>
+      <c r="J5" s="1">
+        <v>18955</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Many imporvements to subsumption-based prefix generator.
</commit_message>
<xml_diff>
--- a/Prefixes.xlsx
+++ b/Prefixes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDB9E51-34BD-46F3-85C3-CA386E0C5129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED155091-3798-41C9-BCDB-5768D522B7C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
+    <workbookView xWindow="-30390" yWindow="4620" windowWidth="28950" windowHeight="14595" activeTab="2" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="2unsym" sheetId="3" r:id="rId1"/>
@@ -691,6 +691,12 @@
       <c r="F2" s="1">
         <v>13</v>
       </c>
+      <c r="G2" s="1">
+        <v>15</v>
+      </c>
+      <c r="H2" s="1">
+        <v>41</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -818,6 +824,12 @@
       <c r="E2" s="1">
         <v>7</v>
       </c>
+      <c r="F2" s="1">
+        <v>148</v>
+      </c>
+      <c r="G2" s="1">
+        <v>570</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -919,36 +931,40 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B8" s="1">
-        <f>B4/B5</f>
+        <f>B4/B2</f>
         <v>1</v>
       </c>
       <c r="C8" s="1">
-        <f t="shared" ref="C8:I8" si="0">C4/C5</f>
+        <f t="shared" ref="C8:J8" si="0">C4/C2</f>
         <v>2</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" si="0"/>
-        <v>1.875</v>
+        <v>5</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" si="0"/>
-        <v>1.7407407407407407</v>
+        <v>6.7142857142857144</v>
       </c>
       <c r="F8" s="1">
         <f t="shared" si="0"/>
-        <v>1.5949367088607596</v>
+        <v>3.4054054054054053</v>
       </c>
       <c r="G8" s="1">
         <f t="shared" si="0"/>
-        <v>1.4822888283378746</v>
-      </c>
-      <c r="H8" s="1">
+        <v>2.8631578947368421</v>
+      </c>
+      <c r="H8" s="1" t="e">
         <f t="shared" si="0"/>
-        <v>1.5348437599439955</v>
-      </c>
-      <c r="I8" s="1">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I8" s="1" t="e">
         <f t="shared" si="0"/>
-        <v>1.430792061775285</v>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J8" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
@@ -1046,6 +1062,12 @@
       <c r="H2" s="1">
         <v>68</v>
       </c>
+      <c r="I2" s="1">
+        <v>3090</v>
+      </c>
+      <c r="J2" s="1">
+        <v>6176</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">

</xml_diff>

<commit_message>
Implement equivalent output pruning, making prune one-directional.
</commit_message>
<xml_diff>
--- a/Prefixes.xlsx
+++ b/Prefixes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED155091-3798-41C9-BCDB-5768D522B7C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1404E2A3-9638-482D-B778-C7013E1E06A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28455" yWindow="885" windowWidth="28950" windowHeight="14595" activeTab="2" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="2unsym" sheetId="3" r:id="rId1"/>
@@ -1068,6 +1068,9 @@
       <c r="J2" s="1">
         <v>6176</v>
       </c>
+      <c r="K2" s="1">
+        <v>111307</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">

</xml_diff>